<commit_message>
Adiciona sheet tela_inicial com 13 campos da tela inicial
</commit_message>
<xml_diff>
--- a/dados_projeto/tipos_ordem_template.xlsx
+++ b/dados_projeto/tipos_ordem_template.xlsx
@@ -6,13 +6,14 @@
   <sheets>
     <sheet sheetId="1" name="tipos_ordem" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Texto_ordem" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="tela_inicial" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1349" uniqueCount="221">
   <si>
     <t>tipo_ordem</t>
   </si>
@@ -650,6 +651,123 @@
  FOI COLHIDA LEITURA VISUAL E NETBOOK: 
  OBSERVAÇÃO: 
 </t>
+  </si>
+  <si>
+    <t>obrigatorio</t>
+  </si>
+  <si>
+    <t>Tipo de Ordem</t>
+  </si>
+  <si>
+    <t>(50 tipos)</t>
+  </si>
+  <si>
+    <t>Selecione o tipo</t>
+  </si>
+  <si>
+    <t>cliente</t>
+  </si>
+  <si>
+    <t>Cliente</t>
+  </si>
+  <si>
+    <t>(~140 clientes)</t>
+  </si>
+  <si>
+    <t>Selecione o cliente</t>
+  </si>
+  <si>
+    <t>Ordem</t>
+  </si>
+  <si>
+    <t>Número da Ordem de Serviço</t>
+  </si>
+  <si>
+    <t>uc</t>
+  </si>
+  <si>
+    <t>UC</t>
+  </si>
+  <si>
+    <t>Número da UC</t>
+  </si>
+  <si>
+    <t>municipio</t>
+  </si>
+  <si>
+    <t>Município</t>
+  </si>
+  <si>
+    <t>(lista de municípios)</t>
+  </si>
+  <si>
+    <t>Selecione o município</t>
+  </si>
+  <si>
+    <t>apr</t>
+  </si>
+  <si>
+    <t>APR</t>
+  </si>
+  <si>
+    <t>Número APR</t>
+  </si>
+  <si>
+    <t>pre_apr</t>
+  </si>
+  <si>
+    <t>PRE APR</t>
+  </si>
+  <si>
+    <t>Número PRE APR</t>
+  </si>
+  <si>
+    <t>notificado</t>
+  </si>
+  <si>
+    <t>Notificado</t>
+  </si>
+  <si>
+    <t>muck_bq</t>
+  </si>
+  <si>
+    <t>Muck B&amp;Q</t>
+  </si>
+  <si>
+    <t>placa</t>
+  </si>
+  <si>
+    <t>Placa</t>
+  </si>
+  <si>
+    <t>Placa do veículo</t>
+  </si>
+  <si>
+    <t>tecnicos</t>
+  </si>
+  <si>
+    <t>Técnico(s)</t>
+  </si>
+  <si>
+    <t>Nome do(s) técnico(s)</t>
+  </si>
+  <si>
+    <t>data_hora</t>
+  </si>
+  <si>
+    <t>Data/Hora</t>
+  </si>
+  <si>
+    <t>Data e hora (automático)</t>
+  </si>
+  <si>
+    <t>observacao</t>
+  </si>
+  <si>
+    <t>Observação</t>
+  </si>
+  <si>
+    <t>Observação geral</t>
   </si>
 </sst>
 </file>
@@ -5622,4 +5740,473 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>184</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>185</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" t="s">
+        <v>188</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>189</v>
+      </c>
+      <c r="J3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s">
+        <v>194</v>
+      </c>
+      <c r="J5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>197</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" t="s">
+        <v>198</v>
+      </c>
+      <c r="J6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>199</v>
+      </c>
+      <c r="C7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" t="s">
+        <v>201</v>
+      </c>
+      <c r="J7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" t="s">
+        <v>203</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>64</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" t="s">
+        <v>204</v>
+      </c>
+      <c r="J8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>205</v>
+      </c>
+      <c r="C9" t="s">
+        <v>206</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>207</v>
+      </c>
+      <c r="C10" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" t="s">
+        <v>208</v>
+      </c>
+      <c r="J10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11" t="s">
+        <v>210</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" t="s">
+        <v>211</v>
+      </c>
+      <c r="J11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>212</v>
+      </c>
+      <c r="C12" t="s">
+        <v>213</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" t="s">
+        <v>214</v>
+      </c>
+      <c r="J12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>215</v>
+      </c>
+      <c r="C13" t="s">
+        <v>216</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" t="s">
+        <v>217</v>
+      </c>
+      <c r="J13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" t="s">
+        <v>219</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" t="s">
+        <v>220</v>
+      </c>
+      <c r="J14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: ajustes de UI - remove textos, botões fixos, date width mobile, selects mais altos
</commit_message>
<xml_diff>
--- a/dados_projeto/tipos_ordem_template.xlsx
+++ b/dados_projeto/tipos_ordem_template.xlsx
@@ -1,19 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A22DCE-F275-4F79-BCB6-3A139F4DF395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="tipos_ordem" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Texto_ordem" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="tela_inicial" state="visible" r:id="rId6"/>
+    <sheet name="tipos_ordem" sheetId="1" r:id="rId1"/>
+    <sheet name="Texto_ordem" sheetId="2" r:id="rId2"/>
+    <sheet name="tela_inicial" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1349" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="220">
   <si>
     <t>tipo_ordem</t>
   </si>
@@ -659,131 +676,130 @@
     <t>Tipo de Ordem</t>
   </si>
   <si>
-    <t>(50 tipos)</t>
-  </si>
-  <si>
     <t>Selecione o tipo</t>
   </si>
   <si>
-    <t>cliente</t>
-  </si>
-  <si>
-    <t>Cliente</t>
-  </si>
-  <si>
-    <t>(~140 clientes)</t>
-  </si>
-  <si>
-    <t>Selecione o cliente</t>
-  </si>
-  <si>
-    <t>Ordem</t>
-  </si>
-  <si>
-    <t>Número da Ordem de Serviço</t>
-  </si>
-  <si>
     <t>uc</t>
   </si>
   <si>
     <t>UC</t>
   </si>
   <si>
-    <t>Número da UC</t>
-  </si>
-  <si>
     <t>municipio</t>
   </si>
   <si>
     <t>Município</t>
   </si>
   <si>
-    <t>(lista de municípios)</t>
-  </si>
-  <si>
-    <t>Selecione o município</t>
-  </si>
-  <si>
-    <t>apr</t>
-  </si>
-  <si>
-    <t>APR</t>
-  </si>
-  <si>
-    <t>Número APR</t>
-  </si>
-  <si>
-    <t>pre_apr</t>
-  </si>
-  <si>
-    <t>PRE APR</t>
-  </si>
-  <si>
-    <t>Número PRE APR</t>
-  </si>
-  <si>
     <t>notificado</t>
   </si>
   <si>
     <t>Notificado</t>
   </si>
   <si>
-    <t>muck_bq</t>
-  </si>
-  <si>
-    <t>Muck B&amp;Q</t>
-  </si>
-  <si>
     <t>placa</t>
   </si>
   <si>
     <t>Placa</t>
   </si>
   <si>
-    <t>Placa do veículo</t>
-  </si>
-  <si>
-    <t>tecnicos</t>
-  </si>
-  <si>
-    <t>Técnico(s)</t>
-  </si>
-  <si>
-    <t>Nome do(s) técnico(s)</t>
-  </si>
-  <si>
-    <t>data_hora</t>
-  </si>
-  <si>
-    <t>Data/Hora</t>
-  </si>
-  <si>
-    <t>Data e hora (automático)</t>
-  </si>
-  <si>
-    <t>observacao</t>
-  </si>
-  <si>
-    <t>Observação</t>
-  </si>
-  <si>
-    <t>Observação geral</t>
+    <t>data</t>
+  </si>
+  <si>
+    <t>hora_inicio</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Inicio</t>
+  </si>
+  <si>
+    <t>DATA</t>
+  </si>
+  <si>
+    <t>HORA</t>
+  </si>
+  <si>
+    <t>NUMBER</t>
+  </si>
+  <si>
+    <t>os</t>
+  </si>
+  <si>
+    <t>OS</t>
+  </si>
+  <si>
+    <t>linha_campo</t>
+  </si>
+  <si>
+    <t>hora_fim</t>
+  </si>
+  <si>
+    <t>Fim</t>
+  </si>
+  <si>
+    <t>ANDRE DE SOUSA CARVALHO,ANTONIO MAURIELLTON DE ARAUJO MARTINS,BERKSON EVANGELISTA DE OLIVEIRA,CARLOS CRISTIANO DO NASCIMENTO SILVA,DIEGO DA SILVA DE LIMA,DOUGLAS MONTEIRO DE ABREU,FRANCISCO ADRIANO DE SOUSA VIANA,JOSE DOGIVAN DA SILVA,LEANDRO OLIVEIRA SOUSA,MARCIO JOHNNATAN CHAGAS CAETANO,RENATO RODRIGUES VIEIRA,VALDI DOS SANTOS VIANA FILHO</t>
+  </si>
+  <si>
+    <t>ACARAPE,AQUIRAZ,ARACOIABA,ARATUBA,BARREIRA,BATURITE,BEBERIBE,CAPISTRANO,CASCAVEL,CAUCAIA,CHOROZINHO,EUSÉBIO,FORTALEZA,GUAIUBA,GUARAMIRANGA,HORIZONTE,ITAITINGA,ITAPIUNA,MARACANAU,MARANGUAPE,MULUNGU,OCARA,PACAJUS,PACATUBA,PACOTI,PALMACIA,PINDORETAMA,REDENCAO,SAO GONCALO</t>
+  </si>
+  <si>
+    <t>Lider</t>
+  </si>
+  <si>
+    <t>Parceiro</t>
+  </si>
+  <si>
+    <t>lider</t>
+  </si>
+  <si>
+    <t>parceiro</t>
+  </si>
+  <si>
+    <t>RHS6G02,RIE0D84,RIH3H88,SDZ7E43,SDZ9B15,SDZ9B16,SRT8J10,SRW6J12,SRW6J13,SRW6J41,TCI4F69,TUL0I49</t>
+  </si>
+  <si>
+    <t>Selecione</t>
+  </si>
+  <si>
+    <t>Ordem de Serviço</t>
+  </si>
+  <si>
+    <t>N° UC</t>
+  </si>
+  <si>
+    <t>N° Placa</t>
+  </si>
+  <si>
+    <t>ADEQUACAO SMF,AFERIÇÃO DE MEDIDOR,AFERIÇÃO MEDIDOR CLIENTE LIVRE,COLHER LEITURA,CORTE DE UC POR DEF TECNICO,CORTE DEFINITIVO A PEDIDO,CORTE POR FALTA DE PAGAMENTO,DESLIG.PROG.MANUTENÇÃO,DESLOCAMENTO DE SUBESTAÇÃO,DISPON. SAIDA SERIAL MEDIDOR,EXECUÇÃO DE MUDANÇA DE TARIFA,EXECUCAO DO ACRESCIMO DE POTENCIA,EXECUCAO DO DECRESCIMO DE POTENCIA,GRANDES CLIENTES SELO ROMPIDO,GRANDES CLIENTES SEM MEDIÇÃO,INSPECAO UC CORTADA I15,INSPECAO UC CORTADA I180,INSPECAO UC CORTADA I30,INSPECAO UC CORTADA I90,INSTALACAO DO DISPLAY,LIBERACAO DE PULSO,LIGAÇÃO NOVA ISOLADA,LIGACAO NOVA MEDIA TENSAO,LIGACAO NOVA MT - CLIENTE LIVRE,LIGAÇÃO NOVA SIMULTÂNEA,RELIGACAO NORMAL RURAL,RELIGAÇÃO NORMAL URBANA,RESELAR MEDICAO,RESSERVICO,RETIRAR EQUIPAMENTOS,RETIRAR RAMAL,SERVIÇO ESPECIAL OPERAÇÃO GRUPO A,SUBST. DE EQUIPAMENTO DE MEDICAO,SUBST. MEDIDOR A PEDIDO,SUBST. MEDIDOR INICIATIVA COELCE,SUBSTITUIÇÃO DA BATERIA DO MEDIDOR,SUBSTITUIÇÃO DE DISPLAY,TELEMEDIÇÃO MANUTENÇÃO,TELEMEDIÇÃO MANUTENÇÃO CLIENTE LIVRE,TELEMEDIÇÃO MANUTENÇÃO LOTE,VISITA TECNICA GRUPO A,VISTORIA DA UC,VISTORIA GERAÇÃO DISTRIBUIDA</t>
+  </si>
+  <si>
+    <t>Etapa</t>
+  </si>
+  <si>
+    <t>Iniciais</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -806,9 +822,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1147,9 +1169,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M108"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -5593,16 +5615,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M108"/>
+  <autoFilter ref="A1:M108" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="120" customWidth="1"/>
@@ -5738,475 +5760,485 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J14"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="1" max="2" width="8" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="10" width="13.140625" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>205</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K2" t="s">
+        <v>212</v>
+      </c>
+      <c r="L2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>210</v>
+      </c>
+      <c r="E3" t="s">
+        <v>208</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" t="s">
+        <v>205</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K3" t="s">
+        <v>212</v>
+      </c>
+      <c r="L3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>206</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K4" t="s">
+        <v>212</v>
+      </c>
+      <c r="L4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C5" s="3">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" t="s">
+        <v>186</v>
+      </c>
+      <c r="F5" t="s">
+        <v>199</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K5" t="s">
+        <v>214</v>
+      </c>
+      <c r="L5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="3">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K6" t="s">
+        <v>213</v>
+      </c>
+      <c r="L6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C7" s="3">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K7" t="s">
+        <v>212</v>
+      </c>
+      <c r="L7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C8" s="3">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>191</v>
+      </c>
+      <c r="E8" t="s">
+        <v>192</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K8" t="s">
+        <v>215</v>
+      </c>
+      <c r="L8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C9" s="3">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>193</v>
+      </c>
+      <c r="E9" t="s">
+        <v>195</v>
+      </c>
+      <c r="F9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K9" t="s">
+        <v>212</v>
+      </c>
+      <c r="L9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C10" s="3">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>194</v>
+      </c>
+      <c r="E10" t="s">
+        <v>196</v>
+      </c>
+      <c r="F10" t="s">
+        <v>198</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>18</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K10" t="s">
+        <v>212</v>
+      </c>
+      <c r="L10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C11" s="3">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>203</v>
+      </c>
+      <c r="E11" t="s">
+        <v>204</v>
+      </c>
+      <c r="F11" t="s">
+        <v>198</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K11" t="s">
+        <v>212</v>
+      </c>
+      <c r="L11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C12" s="3">
+        <v>7</v>
+      </c>
+      <c r="D12" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E12" t="s">
         <v>183</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F12" t="s">
         <v>27</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G12" t="s">
+        <v>216</v>
+      </c>
+      <c r="H12" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K12" t="s">
         <v>184</v>
       </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" t="s">
-        <v>185</v>
-      </c>
-      <c r="J2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>186</v>
-      </c>
-      <c r="C3" t="s">
-        <v>187</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" t="s">
-        <v>188</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I3" t="s">
-        <v>189</v>
-      </c>
-      <c r="J3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>190</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" t="s">
-        <v>191</v>
-      </c>
-      <c r="J4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>192</v>
-      </c>
-      <c r="C5" t="s">
-        <v>193</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" t="s">
-        <v>194</v>
-      </c>
-      <c r="J5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C6" t="s">
-        <v>196</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s">
-        <v>197</v>
-      </c>
-      <c r="F6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I6" t="s">
-        <v>198</v>
-      </c>
-      <c r="J6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>199</v>
-      </c>
-      <c r="C7" t="s">
-        <v>200</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" t="s">
-        <v>201</v>
-      </c>
-      <c r="J7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>202</v>
-      </c>
-      <c r="C8" t="s">
-        <v>203</v>
-      </c>
-      <c r="D8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" t="s">
-        <v>204</v>
-      </c>
-      <c r="J8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>205</v>
-      </c>
-      <c r="C9" t="s">
-        <v>206</v>
-      </c>
-      <c r="D9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>207</v>
-      </c>
-      <c r="C10" t="s">
-        <v>208</v>
-      </c>
-      <c r="D10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" t="s">
-        <v>208</v>
-      </c>
-      <c r="J10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>209</v>
-      </c>
-      <c r="C11" t="s">
-        <v>210</v>
-      </c>
-      <c r="D11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" t="s">
-        <v>211</v>
-      </c>
-      <c r="J11" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>212</v>
-      </c>
-      <c r="C12" t="s">
-        <v>213</v>
-      </c>
-      <c r="D12" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" t="s">
-        <v>214</v>
-      </c>
-      <c r="J12" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>215</v>
-      </c>
-      <c r="C13" t="s">
-        <v>216</v>
-      </c>
-      <c r="D13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" t="s">
-        <v>217</v>
-      </c>
-      <c r="J13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>218</v>
-      </c>
-      <c r="C14" t="s">
-        <v>219</v>
-      </c>
-      <c r="D14" t="s">
-        <v>55</v>
-      </c>
-      <c r="E14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" t="s">
-        <v>220</v>
-      </c>
-      <c r="J14" t="s">
-        <v>64</v>
+      <c r="L12" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implementar campos de retorno da aba corte (CORTE, DESLIG, LIGACAO NOVA MT)
</commit_message>
<xml_diff>
--- a/dados_projeto/tipos_ordem_template.xlsx
+++ b/dados_projeto/tipos_ordem_template.xlsx
@@ -3,14 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A22DCE-F275-4F79-BCB6-3A139F4DF395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87223FDF-654E-413F-B76B-B686D0D9FD93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tipos_ordem" sheetId="1" r:id="rId1"/>
     <sheet name="Texto_ordem" sheetId="2" r:id="rId2"/>
     <sheet name="tela_inicial" sheetId="3" r:id="rId3"/>
+    <sheet name="corte" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="263">
   <si>
     <t>tipo_ordem</t>
   </si>
@@ -782,6 +783,135 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>situacao_corte</t>
+  </si>
+  <si>
+    <t>CLIENTE CORTADO,CLIENTE VISITADO CONTA PAGA,CLIENTE NAO PERMITIU O CORTE,SEM ACESSO PARA EXECUTAR O CORTE</t>
+  </si>
+  <si>
+    <t>NÃO TEM</t>
+  </si>
+  <si>
+    <t>DESLI.PROG.MANUTENÇÃO</t>
+  </si>
+  <si>
+    <t>desligamento</t>
+  </si>
+  <si>
+    <t>DESLIGAMENTO EXECUTADO,CLIENTE CANCELOU DESLIGAMENTO,SEM ACESSO,NAO EXECUTADO PENDENCIA CLIENTE,NAO EXECUTADO PENDENCIA ENEL</t>
+  </si>
+  <si>
+    <t>acesso_desligamento</t>
+  </si>
+  <si>
+    <t>NAO</t>
+  </si>
+  <si>
+    <t>CLIENTE CANCELOU DESLIGAMENTO,SEM ACESSO,NAO EXECUTADO PENDENCIA CLIENTE,NAO EXECUTADO PENDENCIA ENEL</t>
+  </si>
+  <si>
+    <t>retorno_ligacao</t>
+  </si>
+  <si>
+    <t>obra</t>
+  </si>
+  <si>
+    <t>VISTORIA, VISTORIA + LIGAÇÃO</t>
+  </si>
+  <si>
+    <t>ACOPLADA,CUBICULO,SEMI-DIRETA,DIRETA</t>
+  </si>
+  <si>
+    <t>tipo_medicao</t>
+  </si>
+  <si>
+    <t>status_medicao</t>
+  </si>
+  <si>
+    <t>ponto_de_entrega</t>
+  </si>
+  <si>
+    <t>medidor_bt</t>
+  </si>
+  <si>
+    <t>qtd_medidor_bt</t>
+  </si>
+  <si>
+    <t>COM MEDIDOR BT,SEM MEDIDOR BT</t>
+  </si>
+  <si>
+    <t>COM MEDIDOR BT</t>
+  </si>
+  <si>
+    <t>CONCLUIDA,NAO CONCLUIDA</t>
+  </si>
+  <si>
+    <t>COM MEDICAO,SEM MEDICAO</t>
+  </si>
+  <si>
+    <t>DE ACORDO,EM DESACORDO,NÃO CONSTRUIDO</t>
+  </si>
+  <si>
+    <t>REGULAR,IRREGULAR,SEM ACESSO</t>
+  </si>
+  <si>
+    <t>acesso_medicao</t>
+  </si>
+  <si>
+    <t>acesso_ponto_de_entrega</t>
+  </si>
+  <si>
+    <t>IRREGULAR,SEM ACESSO</t>
+  </si>
+  <si>
+    <t>situação</t>
+  </si>
+  <si>
+    <t>Desligamento</t>
+  </si>
+  <si>
+    <t>Descreva o Problema</t>
+  </si>
+  <si>
+    <t>Executado</t>
+  </si>
+  <si>
+    <t>Obra</t>
+  </si>
+  <si>
+    <t>Mediçao</t>
+  </si>
+  <si>
+    <t>Status Medição</t>
+  </si>
+  <si>
+    <t>Ponto de Entrega</t>
+  </si>
+  <si>
+    <t>Medidor de BT</t>
+  </si>
+  <si>
+    <t>Quantidade</t>
+  </si>
+  <si>
+    <t>Acesso</t>
+  </si>
+  <si>
+    <t>ligacao</t>
+  </si>
+  <si>
+    <t>VISTORIA,VISTORIA + LIGAÇÃO,LIGAÇÃO</t>
+  </si>
+  <si>
+    <t>LIGAÇÃO</t>
+  </si>
+  <si>
+    <t>Ligação</t>
+  </si>
+  <si>
+    <t>LIGACAO NOVA MEDIA TENSAO,LIGACAO NOVA MT - CLIENTE LIVRE</t>
   </si>
 </sst>
 </file>
@@ -822,7 +952,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -830,6 +960,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6241,4 +6377,542 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{680B7669-68A3-4E37-A5EB-FC8FE51D74EE}">
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8" style="3" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" customWidth="1"/>
+    <col min="7" max="7" width="40.7109375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="34.85546875" style="4" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" t="s">
+        <v>220</v>
+      </c>
+      <c r="E2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="K2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" t="s">
+        <v>224</v>
+      </c>
+      <c r="E3" t="s">
+        <v>248</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="K3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E4" t="s">
+        <v>249</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="K4" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E5" t="s">
+        <v>250</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="K5" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D6" t="s">
+        <v>230</v>
+      </c>
+      <c r="E6" t="s">
+        <v>251</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K6" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E7" t="s">
+        <v>252</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3">
+        <v>3</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D8" t="s">
+        <v>234</v>
+      </c>
+      <c r="E8" t="s">
+        <v>253</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>5</v>
+      </c>
+      <c r="B9" s="3">
+        <v>3</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" t="s">
+        <v>235</v>
+      </c>
+      <c r="E9" t="s">
+        <v>254</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K9" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D10" t="s">
+        <v>236</v>
+      </c>
+      <c r="E10" t="s">
+        <v>255</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>7</v>
+      </c>
+      <c r="B11" s="3">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D11" t="s">
+        <v>237</v>
+      </c>
+      <c r="E11" t="s">
+        <v>256</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="K11" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3">
+        <v>5</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D12" t="s">
+        <v>244</v>
+      </c>
+      <c r="E12" t="s">
+        <v>257</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K12" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>9</v>
+      </c>
+      <c r="B13" s="3">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D13" t="s">
+        <v>245</v>
+      </c>
+      <c r="E13" t="s">
+        <v>249</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="K13" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>2</v>
+      </c>
+      <c r="B14" s="3">
+        <v>2</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D14" t="s">
+        <v>258</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="K14" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>3</v>
+      </c>
+      <c r="B15" s="3">
+        <v>3</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="K15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add descricao field to all order types and remove dead composicao state
</commit_message>
<xml_diff>
--- a/dados_projeto/tipos_ordem_template.xlsx
+++ b/dados_projeto/tipos_ordem_template.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965EB466-C5F9-4916-811C-F8E61901D602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCA5E41D-720E-4AB7-98C2-5ACCE3665CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="afericao" sheetId="4" r:id="rId1"/>
+    <sheet name="campos_retorno" sheetId="4" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="37">
   <si>
     <t>tipo_ordem</t>
   </si>
@@ -66,18 +66,6 @@
     <t>SELECT</t>
   </si>
   <si>
-    <t>TOI</t>
-  </si>
-  <si>
-    <t>numero_toi</t>
-  </si>
-  <si>
-    <t>APLICADO TOI</t>
-  </si>
-  <si>
-    <t>NAO FOI APLICADO TOI</t>
-  </si>
-  <si>
     <t>linha_campo</t>
   </si>
   <si>
@@ -87,71 +75,77 @@
     <t>NAO</t>
   </si>
   <si>
-    <t>AFERIÇAO DE MEDIDOR / AFERIÇAO DE MEDIDOR CLIENTE LIVRE</t>
-  </si>
-  <si>
-    <t>medidor_afericao</t>
-  </si>
-  <si>
-    <t>Medidor</t>
-  </si>
-  <si>
-    <t>Motivo_cancel_afercicao</t>
-  </si>
-  <si>
-    <t>Motivo Cancelamento</t>
-  </si>
-  <si>
-    <t>TEXTO</t>
-  </si>
-  <si>
-    <t>SUBSTITUIDO,NAO SUBSTITUIDO</t>
-  </si>
-  <si>
-    <t>NAO SUBSTITUIDO</t>
-  </si>
-  <si>
-    <t>leitura_afericao</t>
-  </si>
-  <si>
-    <t>VISUAL E NETBOOK,APENAS VISUAL,APENAS NOTEBOOK,NAO FOI COLHIDO LEITURA</t>
-  </si>
-  <si>
-    <t>SUBSTITUIDO</t>
-  </si>
-  <si>
-    <t>toi_afericao</t>
-  </si>
-  <si>
-    <t>APLICADO TOI,PERDAS JA APLICOU TOI,NAO FOI APLICADO TOI</t>
-  </si>
-  <si>
-    <t>porque_nao_aplicado_toi</t>
-  </si>
-  <si>
-    <t>N° TOI</t>
-  </si>
-  <si>
-    <t>Leitura</t>
-  </si>
-  <si>
-    <t>NAO FOI COLHIDO LEITURA</t>
-  </si>
-  <si>
-    <t>motivo_nao_colher</t>
-  </si>
-  <si>
-    <t>Porque não foi colhido</t>
-  </si>
-  <si>
-    <t>Porque não foi aplicado TOI</t>
+    <t>TELEMEDIÇÃO MANUTENÇÃO / TELEMEDIÇÃO MANUTENÇÃO CLIENTE LIVRE / TELEMEDIÇÃO MANUTENÇÃO LOTE</t>
+  </si>
+  <si>
+    <t>Executado</t>
+  </si>
+  <si>
+    <t>Motivo</t>
+  </si>
+  <si>
+    <t>NÃO</t>
+  </si>
+  <si>
+    <t>SIM,NAO</t>
+  </si>
+  <si>
+    <t>SEM ACESSO,MEDICAO COM BY-PASS,MEDICAO AVARIADA,OUTRO MOTIVO</t>
+  </si>
+  <si>
+    <t>Descreva Problema</t>
+  </si>
+  <si>
+    <t>TEXT AREA</t>
+  </si>
+  <si>
+    <t>TEXT</t>
+  </si>
+  <si>
+    <t>atendente_com</t>
+  </si>
+  <si>
+    <t>descreva_problema_telemedicao</t>
+  </si>
+  <si>
+    <t>atentende_com</t>
+  </si>
+  <si>
+    <t>CORTE DE UC POR DEF TECNICO</t>
+  </si>
+  <si>
+    <t>corte_por_defeito_tecnico</t>
+  </si>
+  <si>
+    <t>executado_telemedicao</t>
+  </si>
+  <si>
+    <t>descreva_problema_corte_por_defeito_tecnico</t>
+  </si>
+  <si>
+    <t>SEM ACESSO,SOLICITACAO ENEL,CLIENTE NAO PERMITIU,CLIENTE CORRIGIU PROBLEMA,OUTRO PROBLEMA</t>
+  </si>
+  <si>
+    <t>motivo_cancelamento_telemedicao</t>
+  </si>
+  <si>
+    <t>motivo_cancelamento_corte_por_defeito_tecnico</t>
+  </si>
+  <si>
+    <t>SEM ACESSO,OUTRO PROBLEMA</t>
+  </si>
+  <si>
+    <t>realizado_telemedicao</t>
+  </si>
+  <si>
+    <t>O que foi realizado</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,14 +158,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -194,9 +180,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -206,10 +191,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -549,31 +530,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{680B7669-68A3-4E37-A5EB-FC8FE51D74EE}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" style="3" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="57.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.7109375" customWidth="1"/>
-    <col min="7" max="7" width="75.85546875" style="4" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+    <col min="1" max="1" width="6.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="44.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="31.42578125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.28515625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" style="3" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -585,16 +566,16 @@
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -602,298 +583,260 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>19</v>
+      <c r="C2" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
+        <v>29</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" t="s">
-        <v>17</v>
+      <c r="K2" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>19</v>
+      <c r="C3" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>17</v>
+      <c r="I3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>19</v>
+      <c r="C4" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K4" t="s">
-        <v>17</v>
+      <c r="I4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>19</v>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="F5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>35</v>
+      <c r="I5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>5</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>19</v>
+      <c r="C6" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K6" t="s">
-        <v>17</v>
+      <c r="I6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3">
-        <v>6</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="A7" s="2">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D7" t="s">
+      <c r="H7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K7" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>19</v>
+      <c r="A8" s="2">
+        <v>2</v>
+      </c>
+      <c r="B8" s="2">
+        <v>2</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K8" t="s">
-        <v>17</v>
+      <c r="I8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E10" s="6"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H11" s="3"/>
-    </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F19" s="3"/>
-      <c r="H19" s="3"/>
-    </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F20" s="3"/>
-      <c r="H20" s="3"/>
-    </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F21" s="3"/>
-      <c r="H21" s="3"/>
-    </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F22" s="3"/>
-      <c r="H22" s="3"/>
-    </row>
-    <row r="23" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F23" s="3"/>
-      <c r="H23" s="3"/>
-    </row>
-    <row r="24" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F24" s="3"/>
-      <c r="H24" s="3"/>
-    </row>
-    <row r="25" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F25" s="3"/>
-      <c r="H25" s="3"/>
-    </row>
-    <row r="26" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F26" s="3"/>
-      <c r="H26" s="3"/>
-    </row>
-    <row r="27" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F27" s="3"/>
-      <c r="H27" s="3"/>
-    </row>
-    <row r="28" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F28" s="3"/>
-      <c r="H28" s="3"/>
-    </row>
-    <row r="29" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F29" s="3"/>
-      <c r="H29" s="3"/>
-    </row>
-    <row r="30" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E30" s="4"/>
-      <c r="F30" s="3"/>
-      <c r="H30" s="3"/>
-    </row>
-    <row r="31" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E31" s="4"/>
-      <c r="F31" s="3"/>
-      <c r="H31" s="3"/>
+      <c r="A9" s="2">
+        <v>3</v>
+      </c>
+      <c r="B9" s="2">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>